<commit_message>
Carregando dados de setembro/2026
</commit_message>
<xml_diff>
--- a/upload/partos-2025.xlsx
+++ b/upload/partos-2025.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Export" sheetId="1" r:id="Rce647c9db9b04f02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Export" sheetId="1" r:id="Rc0566934f19142c6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1836,6 +1836,25 @@
     <x:row>
       <x:c t="inlineStr">
         <x:is>
+          <x:t>HJK</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="8">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c s="8">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c s="9">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c s="9">
+        <x:v>35</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c t="inlineStr">
+        <x:is>
           <x:t>HRAD</x:t>
         </x:is>
       </x:c>
@@ -3584,6 +3603,25 @@
     <x:row>
       <x:c t="inlineStr">
         <x:is>
+          <x:t>HRAD</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="8">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c s="8">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c s="9">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c s="9">
+        <x:v>62</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c t="inlineStr">
+        <x:is>
           <x:t>HRJP</x:t>
         </x:is>
       </x:c>
@@ -5332,6 +5370,25 @@
     <x:row>
       <x:c t="inlineStr">
         <x:is>
+          <x:t>HRJP</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="8">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c s="8">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c s="9">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c s="9">
+        <x:v>49</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c t="inlineStr">
+        <x:is>
           <x:t>MOV</x:t>
         </x:is>
       </x:c>
@@ -6862,7 +6919,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c s="9">
-        <x:v>248</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c s="9">
         <x:v>91</x:v>
@@ -7071,10 +7128,29 @@
         <x:v>8</x:v>
       </x:c>
       <x:c s="9">
-        <x:v>280</x:v>
+        <x:v>281</x:v>
       </x:c>
       <x:c s="9">
         <x:v>104</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>MOV</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="8">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c s="8">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c s="9">
+        <x:v>241</x:v>
+      </x:c>
+      <x:c s="9">
+        <x:v>74</x:v>
       </x:c>
     </x:row>
     <x:row/>

</xml_diff>